<commit_message>
data: MI355X MXFP4 EP=1 TP=8 profiling (chat c=64, default max_model_len)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep1_tp8_profiling/decode_breakdown.xlsx
+++ b/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep1_tp8_profiling/decode_breakdown.xlsx
@@ -471,22 +471,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.839</v>
+        <v>14.28</v>
       </c>
       <c r="D2" t="n">
-        <v>3.9</v>
+        <v>5.1</v>
       </c>
       <c r="E2" t="n">
-        <v>17.118</v>
+        <v>19.879</v>
       </c>
       <c r="F2" t="n">
-        <v>6.2</v>
+        <v>7.2</v>
       </c>
       <c r="G2" t="n">
-        <v>13.42761904761905</v>
+        <v>17.31157142857143</v>
       </c>
       <c r="H2" t="n">
-        <v>19.64761904761905</v>
+        <v>23.84204761904762</v>
       </c>
     </row>
     <row r="3">
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6.279</v>
+        <v>5.599</v>
       </c>
       <c r="D3" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>6.220000000000001</v>
+        <v>6.53047619047619</v>
       </c>
     </row>
     <row r="4">
@@ -517,22 +517,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.239</v>
+        <v>5.639</v>
       </c>
       <c r="D4" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>6.239</v>
+        <v>5.639</v>
       </c>
       <c r="F4" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>6.149523809523809</v>
+        <v>6.200904761904762</v>
       </c>
       <c r="H4" t="n">
-        <v>6.149523809523809</v>
+        <v>6.200904761904762</v>
       </c>
     </row>
     <row r="5">
@@ -547,22 +547,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12.399</v>
+        <v>11.279</v>
       </c>
       <c r="D5" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="E5" t="n">
-        <v>12.399</v>
+        <v>11.279</v>
       </c>
       <c r="F5" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="G5" t="n">
-        <v>12.15909523809524</v>
+        <v>11.90390476190476</v>
       </c>
       <c r="H5" t="n">
-        <v>12.15909523809524</v>
+        <v>11.90390476190476</v>
       </c>
     </row>
     <row r="6">
@@ -577,22 +577,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7.599</v>
+        <v>5.679</v>
       </c>
       <c r="D6" t="n">
-        <v>2.7</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>7.599</v>
+        <v>5.679</v>
       </c>
       <c r="F6" t="n">
-        <v>2.7</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>6.877190476190476</v>
+        <v>6.225714285714286</v>
       </c>
       <c r="H6" t="n">
-        <v>6.877190476190476</v>
+        <v>6.225714285714286</v>
       </c>
     </row>
     <row r="7">
@@ -607,22 +607,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7.799</v>
+        <v>6.039</v>
       </c>
       <c r="D7" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="E7" t="n">
-        <v>13.798</v>
+        <v>11.478</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>4.1</v>
       </c>
       <c r="G7" t="n">
-        <v>6.332380952380952</v>
+        <v>6.282809523809523</v>
       </c>
       <c r="H7" t="n">
-        <v>12.64952380952381</v>
+        <v>12.65142857142857</v>
       </c>
     </row>
     <row r="8">
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5.999</v>
+        <v>5.439</v>
       </c>
       <c r="D8" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>6.317142857142857</v>
+        <v>6.368619047619048</v>
       </c>
     </row>
     <row r="9">
@@ -653,22 +653,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6.199</v>
+        <v>5.759</v>
       </c>
       <c r="D9" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="E9" t="n">
-        <v>6.199</v>
+        <v>5.759</v>
       </c>
       <c r="F9" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="G9" t="n">
-        <v>6.214238095238095</v>
+        <v>6.206666666666667</v>
       </c>
       <c r="H9" t="n">
-        <v>6.214238095238095</v>
+        <v>6.206666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -683,22 +683,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>17.399</v>
+        <v>16.959</v>
       </c>
       <c r="D10" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="E10" t="n">
-        <v>25.118</v>
+        <v>23.998</v>
       </c>
       <c r="F10" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="G10" t="n">
-        <v>17.70566666666667</v>
+        <v>17.59342857142857</v>
       </c>
       <c r="H10" t="n">
-        <v>25.38847619047619</v>
+        <v>24.88576190476191</v>
       </c>
     </row>
     <row r="11">
@@ -708,13 +708,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7.719</v>
+        <v>7.039</v>
       </c>
       <c r="D11" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="G11" t="n">
-        <v>7.682809523809524</v>
+        <v>7.292333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -729,22 +729,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.319</v>
+        <v>7.079</v>
       </c>
       <c r="D12" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="E12" t="n">
-        <v>20.517</v>
+        <v>21.197</v>
       </c>
       <c r="F12" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="G12" t="n">
-        <v>6.223761904761904</v>
+        <v>6.441</v>
       </c>
       <c r="H12" t="n">
-        <v>21.37042857142857</v>
+        <v>20.86190476190476</v>
       </c>
     </row>
     <row r="13">
@@ -754,13 +754,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6.239</v>
+        <v>5.679</v>
       </c>
       <c r="D13" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>6.185666666666667</v>
+        <v>6.159</v>
       </c>
     </row>
     <row r="14">
@@ -770,13 +770,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>7.959</v>
+        <v>8.439</v>
       </c>
       <c r="D14" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>8.961</v>
+        <v>8.261904761904763</v>
       </c>
     </row>
     <row r="15">
@@ -791,22 +791,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10.84</v>
+        <v>21.279</v>
       </c>
       <c r="D15" t="n">
-        <v>3.9</v>
+        <v>7.7</v>
       </c>
       <c r="E15" t="n">
-        <v>17.159</v>
+        <v>26.958</v>
       </c>
       <c r="F15" t="n">
-        <v>6.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>11.41642857142857</v>
+        <v>16.85242857142857</v>
       </c>
       <c r="H15" t="n">
-        <v>17.29176190476191</v>
+        <v>23.0552380952381</v>
       </c>
     </row>
     <row r="16">
@@ -816,13 +816,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6.319</v>
+        <v>5.679</v>
       </c>
       <c r="D16" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>5.875333333333334</v>
+        <v>6.202809523809523</v>
       </c>
     </row>
     <row r="17">
@@ -837,22 +837,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9.359</v>
+        <v>9.839</v>
       </c>
       <c r="D17" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E17" t="n">
-        <v>9.359</v>
+        <v>9.839</v>
       </c>
       <c r="F17" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G17" t="n">
-        <v>9.370428571428571</v>
+        <v>9.433333333333334</v>
       </c>
       <c r="H17" t="n">
-        <v>9.370428571428571</v>
+        <v>9.433333333333334</v>
       </c>
     </row>
     <row r="18">
@@ -867,22 +867,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.799</v>
+        <v>5.679</v>
       </c>
       <c r="D18" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>141.434</v>
+        <v>135.954</v>
       </c>
       <c r="F18" t="n">
-        <v>51.1</v>
+        <v>49</v>
       </c>
       <c r="G18" t="n">
-        <v>6.120952380952381</v>
+        <v>6.145714285714286</v>
       </c>
       <c r="H18" t="n">
-        <v>134.8987619047619</v>
+        <v>136.3901428571429</v>
       </c>
     </row>
     <row r="19">
@@ -892,13 +892,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.759</v>
+        <v>5.68</v>
       </c>
       <c r="D19" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>6.191428571428572</v>
+        <v>6.248571428571428</v>
       </c>
     </row>
     <row r="20">
@@ -908,13 +908,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.159</v>
+        <v>5.719</v>
       </c>
       <c r="D20" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="G20" t="n">
-        <v>6.098095238095238</v>
+        <v>6.321</v>
       </c>
     </row>
     <row r="21">
@@ -924,13 +924,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.799</v>
+        <v>9.879</v>
       </c>
       <c r="D21" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="G21" t="n">
-        <v>10.79528571428571</v>
+        <v>9.458095238095238</v>
       </c>
     </row>
     <row r="22">
@@ -940,13 +940,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>69.35899999999999</v>
+        <v>66.71899999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G22" t="n">
-        <v>65.23161904761905</v>
+        <v>66.29852380952381</v>
       </c>
     </row>
     <row r="23">
@@ -956,13 +956,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.199</v>
+        <v>6.919</v>
       </c>
       <c r="D23" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="G23" t="n">
-        <v>6.204714285714286</v>
+        <v>6.768571428571428</v>
       </c>
     </row>
     <row r="24">
@@ -972,13 +972,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>37.36</v>
+        <v>35.359</v>
       </c>
       <c r="D24" t="n">
-        <v>13.5</v>
+        <v>12.7</v>
       </c>
       <c r="G24" t="n">
-        <v>34.25666666666667</v>
+        <v>35.14966666666667</v>
       </c>
     </row>
     <row r="25">
@@ -989,7 +989,7 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>276.939</v>
+        <v>277.659</v>
       </c>
       <c r="D25" t="n">
         <v>100</v>
@@ -999,7 +999,7 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>272.0170476190476</v>
+        <v>281.6570476190476</v>
       </c>
       <c r="H25" t="inlineStr"/>
     </row>
@@ -1080,51 +1080,51 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>69.35899999999999</v>
+        <v>66.71899999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>69.35899999999999</v>
+        <v>66.71899999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>void ck::kernel_moe_mxgemm&lt;ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 64, 32, 32, 128, 16, 16, 16, 16, 2, 2, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 4, 1, 16&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;, false, (ck::InMemoryDataOperationEnum)1, 1, (ck::TailNumber)0&gt;(ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 64, 32, 32, 128, 16, 16, 16, 16, 2, 2, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 4, 1, 16&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;::Argument)</t>
+          <t>void aiter::reduce_scatter_cross_device_store&lt;std::bfloat16_t, 8&gt;(aiter::RankData*, aiter::RankSignals, aiter::Signal*, int, int)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>37.36</v>
+        <v>35.559</v>
       </c>
       <c r="D3" t="n">
-        <v>37.36</v>
+        <v>17.779</v>
       </c>
       <c r="E3" t="n">
-        <v>13.5</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>void aiter::reduce_scatter_cross_device_store&lt;std::bfloat16_t, 8&gt;(aiter::RankData*, aiter::RankSignals, aiter::Signal*, int, int)</t>
+          <t>void ck::kernel_moe_mxgemm&lt;ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 64, 32, 32, 128, 16, 16, 16, 16, 2, 2, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 4, 1, 16&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;, false, (ck::InMemoryDataOperationEnum)1, 1, (ck::TailNumber)0&gt;(ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 64, 32, 32, 128, 16, 16, 16, 16, 2, 2, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 8, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 4, 1, 16&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;::Argument)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>21.679</v>
+        <v>35.359</v>
       </c>
       <c r="D4" t="n">
-        <v>10.84</v>
+        <v>35.359</v>
       </c>
       <c r="E4" t="n">
-        <v>7.8</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="5">
@@ -1137,13 +1137,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>17.399</v>
+        <v>16.959</v>
       </c>
       <c r="D5" t="n">
-        <v>17.399</v>
+        <v>16.959</v>
       </c>
       <c r="E5" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="6">
@@ -1156,51 +1156,51 @@
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>16.998</v>
+        <v>16.798</v>
       </c>
       <c r="D6" t="n">
-        <v>8.499000000000001</v>
+        <v>8.398999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>void aiter::local_device_load_rmsnorm&lt;std::bfloat16_t, 512, 2&gt;(aiter::RankSignals, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, float, int, int, int)</t>
+          <t>void ck::kernel_gemm_xdl_cshuffle_v3_multi_d_b_preshuffle&lt;ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 16, 32, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 16, 1, 8&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;, true, (ck::InMemoryDataOperationEnum)0, 2, (ck::TailNumber)1&gt;(ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 16, 32, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 16, 1, 8&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;::Argument)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>12.598</v>
+        <v>11.279</v>
       </c>
       <c r="D7" t="n">
-        <v>6.299</v>
+        <v>11.279</v>
       </c>
       <c r="E7" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>void ck::kernel_gemm_xdl_cshuffle_v3_multi_d_b_preshuffle&lt;ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 16, 32, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 16, 1, 8&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;, true, (ck::InMemoryDataOperationEnum)0, 2, (ck::TailNumber)1&gt;(ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 16, 32, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 16, 1, 8&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;::Argument)</t>
+          <t>void aiter::local_device_load_rmsnorm&lt;std::bfloat16_t, 512, 2&gt;(aiter::RankSignals, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, float, int, int, int)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>12.399</v>
+        <v>11.278</v>
       </c>
       <c r="D8" t="n">
-        <v>12.399</v>
+        <v>5.639</v>
       </c>
       <c r="E8" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="9">
@@ -1213,13 +1213,13 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>9.359</v>
+        <v>9.839</v>
       </c>
       <c r="D9" t="n">
-        <v>9.359</v>
+        <v>9.839</v>
       </c>
       <c r="E9" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="10">
@@ -1232,32 +1232,32 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>7.959</v>
+        <v>8.439</v>
       </c>
       <c r="D10" t="n">
-        <v>7.959</v>
+        <v>8.439</v>
       </c>
       <c r="E10" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>void ck::kernel_gemm_xdl_cshuffle_v3_multi_d_b_preshuffle&lt;ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 32, 16, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 32, 1, 4&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;, true, (ck::InMemoryDataOperationEnum)0, 2, (ck::TailNumber)0&gt;(ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 32, 16, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 32, 1, 4&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;::Argument)</t>
+          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_64_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>7.799</v>
+        <v>7.079</v>
       </c>
       <c r="D11" t="n">
-        <v>7.799</v>
+        <v>7.079</v>
       </c>
       <c r="E11" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="12">
@@ -1270,184 +1270,184 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>7.719</v>
+        <v>7.039</v>
       </c>
       <c r="D12" t="n">
-        <v>7.719</v>
+        <v>7.039</v>
       </c>
       <c r="E12" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>_fused_rms_fp8_group_quant_kernel</t>
+          <t>void ck::kernel_gemm_xdl_cshuffle_v3_multi_d_b_preshuffle&lt;ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 32, 16, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 32, 1, 4&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;, true, (ck::InMemoryDataOperationEnum)0, 2, (ck::TailNumber)0&gt;(ck::GridwiseGemmMultiD_xdl_cshuffle_v3_b_preshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f8_fnuz_t, ck::f8_fnuz_t, float, float, ck::Tuple&lt;float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MultiplyMultiply, (ck::tensor_operation::device::GemmSpecialization)0, 128, 32, 16, 512, 16, 16, 16, 16, 1, 1, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, ck::Sequence&lt;32, 4, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 0, 1, 1, ck::Sequence&lt;1, 32, 1, 4&gt;, ck::Sequence&lt;4, 4, 1&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)0, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t, ck::f8_fnuz_t&gt;::Argument)</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>7.599</v>
+        <v>6.039</v>
       </c>
       <c r="D13" t="n">
-        <v>7.599</v>
+        <v>6.039</v>
       </c>
       <c r="E13" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_64_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
+          <t>void aiter::fuse_qk_rope_concat_and_cache_mla_per_head_kernel&lt;std::bfloat16_t, _BitInt(8), _BitInt(8), (vllm::Fp8KVCacheDataType)1, (vllm::Fp8KVCacheDataType)1, 8&gt;(std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, _BitInt(8)*, _BitInt(8)*, long const*, long const*, std::bfloat16_t const*, std::bfloat16_t const*, int, int, int, int, int, int, int, int, int, int, int, int, int, int, float const*, float const*, bool, bool)</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>6.319</v>
+        <v>5.759</v>
       </c>
       <c r="D14" t="n">
-        <v>6.319</v>
+        <v>5.759</v>
       </c>
       <c r="E14" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>void aiter::dynamic_per_token_scaled_quant_kernel&lt;std::bfloat16_t, _BitInt(8), 32&gt;(_BitInt(8)*, float*, std::bfloat16_t*, float const*, int, int const*, int)</t>
+          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs)</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>6.239</v>
+        <v>5.719</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>5.719</v>
       </c>
       <c r="E15" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>void aiter::dynamic_per_token_scaled_quant_kernel&lt;std::bfloat16_t, _BitInt(8), 8&gt;(_BitInt(8)*, float*, std::bfloat16_t*, float const*, int, int const*, int)</t>
+          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs)</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>6.239</v>
+        <v>5.68</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>5.68</v>
       </c>
       <c r="E16" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>void aiter::fuse_qk_rope_concat_and_cache_mla_per_head_kernel&lt;std::bfloat16_t, _BitInt(8), _BitInt(8), (vllm::Fp8KVCacheDataType)1, (vllm::Fp8KVCacheDataType)1, 8&gt;(std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, _BitInt(8)*, _BitInt(8)*, long const*, long const*, std::bfloat16_t const*, std::bfloat16_t const*, int, int, int, int, int, int, int, int, int, int, int, int, int, int, float const*, float const*, bool, bool)</t>
+          <t>_fused_rms_fp8_group_quant_kernel</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>6.199</v>
+        <v>5.679</v>
       </c>
       <c r="D17" t="n">
-        <v>6.199</v>
+        <v>5.679</v>
       </c>
       <c r="E17" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs)</t>
+          <t>void aiter::dynamic_per_token_scaled_quant_kernel&lt;std::bfloat16_t, _BitInt(8), 8&gt;(_BitInt(8)*, float*, std::bfloat16_t*, float const*, int, int const*, int)</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>6.159</v>
+        <v>5.679</v>
       </c>
       <c r="D18" t="n">
-        <v>6.159</v>
+        <v>5.679</v>
       </c>
       <c r="E18" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_128_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
+          <t>void aiter::grouped_topk_opt_sort_kernel&lt;c10::BFloat16, float __vector(4), 8, true, true, false&gt;(c10::BFloat16*, c10::BFloat16 const*, float*, int*, unsigned long, int, int, int, int, float)</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>5.999</v>
+        <v>5.679</v>
       </c>
       <c r="D19" t="n">
-        <v>5.999</v>
+        <v>5.679</v>
       </c>
       <c r="E19" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>void aiter::grouped_topk_opt_sort_kernel&lt;c10::BFloat16, float __vector(4), 8, true, true, false&gt;(c10::BFloat16*, c10::BFloat16 const*, float*, int*, unsigned long, int, int, int, int, float)</t>
+          <t>void aiter::dynamic_per_token_scaled_quant_kernel&lt;std::bfloat16_t, _BitInt(8), 32&gt;(_BitInt(8)*, float*, std::bfloat16_t*, float const*, int, int const*, int)</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>5.799</v>
+        <v>5.639</v>
       </c>
       <c r="D20" t="n">
-        <v>5.799</v>
+        <v>5.639</v>
       </c>
       <c r="E20" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, false, false, true&gt; &gt;::Kargs)</t>
+          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_128_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>5.759</v>
+        <v>5.439</v>
       </c>
       <c r="D21" t="n">
-        <v>5.759</v>
+        <v>5.439</v>
       </c>
       <c r="E21" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>